<commit_message>
data(scrapers): synchronize all primary scrapers, update bunker master, and pass 20/20 live smoke tests
</commit_message>
<xml_diff>
--- a/data/commodities/GTRTable19_Figure19.xlsx
+++ b/data/commodities/GTRTable19_Figure19.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdagcc.sharepoint.com/sites/MRP-AMS-TED/Shared Documents/GTR/WebZip Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="368" documentId="8_{5DC5C50C-B9D1-43B8-8139-6A342E8B45D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{735011D3-EF11-47C2-BCB5-29A5D025CF77}"/>
+  <xr:revisionPtr revIDLastSave="396" documentId="8_{5DC5C50C-B9D1-43B8-8139-6A342E8B45D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DCD68E3-E672-4CA4-BDA5-99076DE74552}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4250" uniqueCount="1692">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4252" uniqueCount="1694">
   <si>
     <t>Gulf</t>
   </si>
@@ -5118,7 +5118,13 @@
     <t>09/03/2026</t>
   </si>
   <si>
-    <t>Week ending 09/03/26, number of vessels</t>
+    <t/>
+  </si>
+  <si>
+    <t>09/10/2026</t>
+  </si>
+  <si>
+    <t>Week ending 09/10/26, number of vessels</t>
   </si>
 </sst>
 </file>
@@ -5439,7 +5445,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -5570,6 +5576,7 @@
     <xf numFmtId="9" fontId="16" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5682,215 +5689,215 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$B$1624:$B$1656</c:f>
+              <c:f>Data!$B$1625:$B$1657</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>01/22/2026</c:v>
+                  <c:v>01/29/2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>01/29/2026</c:v>
+                  <c:v>02/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>02/05/2026</c:v>
+                  <c:v>02/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>02/12/2026</c:v>
+                  <c:v>02/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>02/19/2026</c:v>
+                  <c:v>02/26/2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>02/26/2026</c:v>
+                  <c:v>03/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>03/05/2026</c:v>
+                  <c:v>03/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/12/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>04/02/2026</c:v>
+                  <c:v>04/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>04/09/2026</c:v>
+                  <c:v>04/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>04/16/2026</c:v>
+                  <c:v>04/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>04/23/2026</c:v>
+                  <c:v>04/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>04/30/2026</c:v>
+                  <c:v>05/07/2026</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>05/07/2026</c:v>
+                  <c:v>05/14/2026</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>05/14/2026</c:v>
+                  <c:v>05/21/2026</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>05/21/2026</c:v>
+                  <c:v>05/28/2026</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>05/28/2026</c:v>
+                  <c:v>06/04/2026</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>06/04/2026</c:v>
+                  <c:v>06/11/2026</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>06/11/2026</c:v>
+                  <c:v>06/18/2026</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>06/18/2026</c:v>
+                  <c:v>06/25/2026</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>06/25/2026</c:v>
+                  <c:v>07/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>07/02/2026</c:v>
+                  <c:v>07/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>07/09/2026</c:v>
+                  <c:v>07/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>07/16/2026</c:v>
+                  <c:v>07/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>07/23/2026</c:v>
+                  <c:v>07/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>07/30/2026</c:v>
+                  <c:v>08/06/2026</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>08/06/2026</c:v>
+                  <c:v>08/13/2026</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>08/13/2026</c:v>
+                  <c:v>08/20/2026</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>08/20/2026</c:v>
+                  <c:v>08/27/2026</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>08/27/2026</c:v>
+                  <c:v>09/03/2026</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>09/03/2026</c:v>
+                  <c:v>09/10/2026</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$G$1624:$G$1656</c:f>
+              <c:f>Data!$G$1625:$G$1657</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>30</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>29</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>39</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>31</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>28</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>34</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>32</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>40</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>33</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>29</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>30</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>27</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>26</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="15">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="28">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="16">
-                  <c:v>22</c:v>
+                <c:pt idx="29">
+                  <c:v>23</c:v>
                 </c:pt>
-                <c:pt idx="17">
-                  <c:v>25</c:v>
+                <c:pt idx="30">
+                  <c:v>18</c:v>
                 </c:pt>
-                <c:pt idx="18">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>36</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="21">
+                <c:pt idx="31">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="22">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>32</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>33</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>29</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>18</c:v>
-                </c:pt>
                 <c:pt idx="32">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5920,215 +5927,215 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$B$1624:$B$1656</c:f>
+              <c:f>Data!$B$1625:$B$1657</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>01/22/2026</c:v>
+                  <c:v>01/29/2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>01/29/2026</c:v>
+                  <c:v>02/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>02/05/2026</c:v>
+                  <c:v>02/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>02/12/2026</c:v>
+                  <c:v>02/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>02/19/2026</c:v>
+                  <c:v>02/26/2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>02/26/2026</c:v>
+                  <c:v>03/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>03/05/2026</c:v>
+                  <c:v>03/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/12/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>04/02/2026</c:v>
+                  <c:v>04/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>04/09/2026</c:v>
+                  <c:v>04/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>04/16/2026</c:v>
+                  <c:v>04/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>04/23/2026</c:v>
+                  <c:v>04/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>04/30/2026</c:v>
+                  <c:v>05/07/2026</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>05/07/2026</c:v>
+                  <c:v>05/14/2026</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>05/14/2026</c:v>
+                  <c:v>05/21/2026</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>05/21/2026</c:v>
+                  <c:v>05/28/2026</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>05/28/2026</c:v>
+                  <c:v>06/04/2026</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>06/04/2026</c:v>
+                  <c:v>06/11/2026</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>06/11/2026</c:v>
+                  <c:v>06/18/2026</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>06/18/2026</c:v>
+                  <c:v>06/25/2026</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>06/25/2026</c:v>
+                  <c:v>07/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>07/02/2026</c:v>
+                  <c:v>07/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>07/09/2026</c:v>
+                  <c:v>07/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>07/16/2026</c:v>
+                  <c:v>07/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>07/23/2026</c:v>
+                  <c:v>07/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>07/30/2026</c:v>
+                  <c:v>08/06/2026</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>08/06/2026</c:v>
+                  <c:v>08/13/2026</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>08/13/2026</c:v>
+                  <c:v>08/20/2026</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>08/20/2026</c:v>
+                  <c:v>08/27/2026</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>08/27/2026</c:v>
+                  <c:v>09/03/2026</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>09/03/2026</c:v>
+                  <c:v>09/10/2026</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$I$1624:$I$1656</c:f>
+              <c:f>Data!$I$1625:$I$1657</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>44</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>61</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>50</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>40</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>37</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>48</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>58</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>36</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>42</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="13">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="25">
                   <c:v>41</c:v>
                 </c:pt>
-                <c:pt idx="11">
-                  <c:v>33</c:v>
+                <c:pt idx="26">
+                  <c:v>28</c:v>
                 </c:pt>
-                <c:pt idx="12">
-                  <c:v>40</c:v>
+                <c:pt idx="27">
+                  <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="13">
-                  <c:v>42</c:v>
+                <c:pt idx="28">
+                  <c:v>31</c:v>
                 </c:pt>
-                <c:pt idx="14">
-                  <c:v>40</c:v>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="15">
-                  <c:v>48</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>37</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>38</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="19">
+                <c:pt idx="30">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="20">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>37</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>42</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>41</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>31</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>30</c:v>
-                </c:pt>
                 <c:pt idx="31">
-                  <c:v>29</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>32</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6185,215 +6192,215 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$B$1624:$B$1656</c:f>
+              <c:f>Data!$B$1625:$B$1657</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>01/22/2026</c:v>
+                  <c:v>01/29/2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>01/29/2026</c:v>
+                  <c:v>02/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>02/05/2026</c:v>
+                  <c:v>02/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>02/12/2026</c:v>
+                  <c:v>02/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>02/19/2026</c:v>
+                  <c:v>02/26/2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>02/26/2026</c:v>
+                  <c:v>03/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>03/05/2026</c:v>
+                  <c:v>03/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/12/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>04/02/2026</c:v>
+                  <c:v>04/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>04/09/2026</c:v>
+                  <c:v>04/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>04/16/2026</c:v>
+                  <c:v>04/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>04/23/2026</c:v>
+                  <c:v>04/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>04/30/2026</c:v>
+                  <c:v>05/07/2026</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>05/07/2026</c:v>
+                  <c:v>05/14/2026</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>05/14/2026</c:v>
+                  <c:v>05/21/2026</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>05/21/2026</c:v>
+                  <c:v>05/28/2026</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>05/28/2026</c:v>
+                  <c:v>06/04/2026</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>06/04/2026</c:v>
+                  <c:v>06/11/2026</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>06/11/2026</c:v>
+                  <c:v>06/18/2026</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>06/18/2026</c:v>
+                  <c:v>06/25/2026</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>06/25/2026</c:v>
+                  <c:v>07/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>07/02/2026</c:v>
+                  <c:v>07/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>07/09/2026</c:v>
+                  <c:v>07/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>07/16/2026</c:v>
+                  <c:v>07/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>07/23/2026</c:v>
+                  <c:v>07/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>07/30/2026</c:v>
+                  <c:v>08/06/2026</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>08/06/2026</c:v>
+                  <c:v>08/13/2026</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>08/13/2026</c:v>
+                  <c:v>08/20/2026</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>08/20/2026</c:v>
+                  <c:v>08/27/2026</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>08/27/2026</c:v>
+                  <c:v>09/03/2026</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>09/03/2026</c:v>
+                  <c:v>09/10/2026</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$H$1624:$H$1656</c:f>
+              <c:f>Data!$H$1625:$H$1657</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>28.25</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="1">
+                  <c:v>31.25</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>32.25</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>27.25</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="6">
+                  <c:v>31.75</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>31.25</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>32.25</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>27.25</c:v>
-                </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="8">
                   <c:v>31</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>29</c:v>
+                <c:pt idx="9">
+                  <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="10">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>31.75</c:v>
                 </c:pt>
-                <c:pt idx="8">
-                  <c:v>31.25</c:v>
+                <c:pt idx="12">
+                  <c:v>29.25</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>31</c:v>
+                <c:pt idx="13">
+                  <c:v>26.75</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>30</c:v>
+                <c:pt idx="14">
+                  <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="15">
+                  <c:v>24.75</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>22.75</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>23.5</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>26.5</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>25.75</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>20.75</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>20.25</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>20.75</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>22.25</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>23.25</c:v>
+                </c:pt>
+                <c:pt idx="26">
                   <c:v>28</c:v>
                 </c:pt>
-                <c:pt idx="12">
-                  <c:v>31.75</c:v>
+                <c:pt idx="27">
+                  <c:v>22.5</c:v>
                 </c:pt>
-                <c:pt idx="13">
-                  <c:v>29.25</c:v>
+                <c:pt idx="28">
+                  <c:v>19</c:v>
                 </c:pt>
-                <c:pt idx="14">
-                  <c:v>26.75</c:v>
+                <c:pt idx="29">
+                  <c:v>22.5</c:v>
                 </c:pt>
-                <c:pt idx="15">
-                  <c:v>25</c:v>
+                <c:pt idx="30">
+                  <c:v>26</c:v>
                 </c:pt>
-                <c:pt idx="16">
-                  <c:v>24.75</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>22.75</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>23.5</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>26.5</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>25.75</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>20.75</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>20.25</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>20.75</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>22.25</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="26">
+                <c:pt idx="31">
                   <c:v>23.25</c:v>
                 </c:pt>
-                <c:pt idx="27">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>22.5</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>22.5</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>26</c:v>
-                </c:pt>
                 <c:pt idx="32">
-                  <c:v>23.25</c:v>
+                  <c:v>24.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6965,7 +6972,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:X1826"/>
+  <dimension ref="A1:X1829"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="12" bestFit="1" customWidth="1"/>
@@ -6997,13 +7004,13 @@
       <c r="J1" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="58" t="s">
+      <c r="K1" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="58"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="59"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
       <c r="P1" s="3" t="s">
         <v>5</v>
       </c>
@@ -79807,14 +79814,14 @@
         <v>26</v>
       </c>
       <c r="H1598" s="1">
-        <f t="shared" ref="H1598:H1656" si="87">AVERAGE(G1546,G1494,G1442,G1390)</f>
+        <f t="shared" ref="H1598:H1657" si="87">AVERAGE(G1546,G1494,G1442,G1390)</f>
         <v>25.75</v>
       </c>
       <c r="I1598" s="1">
         <v>37</v>
       </c>
       <c r="J1598" s="1">
-        <f t="shared" ref="J1598:J1656" si="88">AVERAGE(I1546,I1494,I1442,I1390)</f>
+        <f t="shared" ref="J1598:J1657" si="88">AVERAGE(I1546,I1494,I1442,I1390)</f>
         <v>39.75</v>
       </c>
       <c r="K1598" s="1">
@@ -82320,7 +82327,7 @@
         <v>20</v>
       </c>
       <c r="F1643" s="1">
-        <f t="shared" ref="F1643:F1656" si="89">AVERAGE(E1591,E1539,E1487,E1435)</f>
+        <f t="shared" ref="F1643:F1657" si="89">AVERAGE(E1591,E1539,E1487,E1435)</f>
         <v>19</v>
       </c>
       <c r="G1643" s="1">
@@ -83088,9 +83095,48 @@
       </c>
     </row>
     <row r="1657" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1657" s="48"/>
-      <c r="C1657" s="1"/>
-      <c r="D1657" s="1"/>
+      <c r="A1657" s="12">
+        <v>46275</v>
+      </c>
+      <c r="B1657" s="48" t="s">
+        <v>1692</v>
+      </c>
+      <c r="C1657" s="1">
+        <v>7</v>
+      </c>
+      <c r="D1657" s="1">
+        <v>16</v>
+      </c>
+      <c r="E1657" s="1">
+        <v>23</v>
+      </c>
+      <c r="F1657" s="1">
+        <f t="shared" si="89"/>
+        <v>27</v>
+      </c>
+      <c r="G1657" s="1">
+        <v>22</v>
+      </c>
+      <c r="H1657" s="1">
+        <f t="shared" si="87"/>
+        <v>24.25</v>
+      </c>
+      <c r="I1657" s="1">
+        <v>49</v>
+      </c>
+      <c r="J1657" s="1">
+        <f t="shared" si="88"/>
+        <v>47.75</v>
+      </c>
+      <c r="K1657" s="1">
+        <v>4</v>
+      </c>
+      <c r="L1657" s="1">
+        <v>7</v>
+      </c>
+      <c r="M1657" s="1">
+        <v>11</v>
+      </c>
       <c r="P1657" s="2" t="s">
         <v>551</v>
       </c>
@@ -83121,7 +83167,7 @@
       <c r="R1659" s="2"/>
     </row>
     <row r="1660" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1660" s="14"/>
+      <c r="B1660" s="48"/>
       <c r="C1660" s="1"/>
       <c r="D1660" s="1"/>
       <c r="P1660" s="2"/>
@@ -83129,7 +83175,7 @@
       <c r="R1660" s="2"/>
     </row>
     <row r="1661" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1661" s="14"/>
+      <c r="B1661" s="48"/>
       <c r="C1661" s="1"/>
       <c r="D1661" s="1"/>
       <c r="P1661" s="2"/>
@@ -83137,50 +83183,23 @@
       <c r="R1661" s="2"/>
     </row>
     <row r="1662" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1662" s="14" t="s">
-        <v>1618</v>
-      </c>
-      <c r="C1662" s="14"/>
-      <c r="D1662" s="14"/>
-      <c r="E1662" s="26">
-        <f>AVERAGE(E1050:E1102)</f>
-        <v>43.075471698113205</v>
-      </c>
-      <c r="F1662" s="26"/>
-      <c r="G1662" s="26">
-        <f>AVERAGE(G1050:G1102)</f>
-        <v>37.433962264150942</v>
-      </c>
-      <c r="H1662" s="26"/>
-      <c r="I1662" s="26">
-        <f>AVERAGE(I1050:I1102)</f>
-        <v>56.113207547169814</v>
-      </c>
+      <c r="B1662" s="48"/>
+      <c r="C1662" s="1"/>
+      <c r="D1662" s="1"/>
       <c r="P1662" s="2"/>
       <c r="Q1662" s="2"/>
       <c r="R1662" s="2"/>
     </row>
     <row r="1663" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1663" s="25" t="s">
-        <v>1619</v>
-      </c>
-      <c r="C1663" s="25"/>
-      <c r="D1663" s="25"/>
-      <c r="E1663" s="1" t="s">
-        <v>1620</v>
-      </c>
-      <c r="G1663" s="1" t="s">
-        <v>1621</v>
-      </c>
-      <c r="I1663" s="1" t="s">
-        <v>1622</v>
-      </c>
+      <c r="B1663" s="14"/>
+      <c r="C1663" s="1"/>
+      <c r="D1663" s="1"/>
       <c r="P1663" s="2"/>
       <c r="Q1663" s="2"/>
       <c r="R1663" s="2"/>
     </row>
     <row r="1664" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1664" s="1"/>
+      <c r="B1664" s="14"/>
       <c r="C1664" s="1"/>
       <c r="D1664" s="1"/>
       <c r="P1664" s="2"/>
@@ -83188,101 +83207,128 @@
       <c r="R1664" s="2"/>
     </row>
     <row r="1665" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1665" s="1"/>
-      <c r="C1665" s="1"/>
-      <c r="D1665" s="1"/>
-      <c r="E1665" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1665" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1665" s="3" t="s">
-        <v>3</v>
+      <c r="B1665" s="14" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C1665" s="14"/>
+      <c r="D1665" s="14"/>
+      <c r="E1665" s="26">
+        <f>AVERAGE(E1050:E1102)</f>
+        <v>43.075471698113205</v>
+      </c>
+      <c r="F1665" s="26"/>
+      <c r="G1665" s="26">
+        <f>AVERAGE(G1050:G1102)</f>
+        <v>37.433962264150942</v>
+      </c>
+      <c r="H1665" s="26"/>
+      <c r="I1665" s="26">
+        <f>AVERAGE(I1050:I1102)</f>
+        <v>56.113207547169814</v>
       </c>
       <c r="P1665" s="2"/>
       <c r="Q1665" s="2"/>
       <c r="R1665" s="2"/>
     </row>
     <row r="1666" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E1666" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1666" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1666" s="39" t="s">
-        <v>1623</v>
-      </c>
-      <c r="L1666" s="1" t="s">
-        <v>1624</v>
+      <c r="B1666" s="25" t="s">
+        <v>1619</v>
+      </c>
+      <c r="C1666" s="25"/>
+      <c r="D1666" s="25"/>
+      <c r="E1666" s="1" t="s">
+        <v>1620</v>
+      </c>
+      <c r="G1666" s="1" t="s">
+        <v>1621</v>
+      </c>
+      <c r="I1666" s="1" t="s">
+        <v>1622</v>
       </c>
       <c r="P1666" s="2"/>
       <c r="Q1666" s="2"/>
       <c r="R1666" s="2"/>
     </row>
     <row r="1667" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1667" s="16" t="s">
-        <v>1625</v>
-      </c>
-      <c r="E1667" s="20">
-        <f>(E1656/E1604)-1</f>
-        <v>-8.333333333333337E-2</v>
-      </c>
-      <c r="F1667" s="20"/>
-      <c r="G1667" s="20">
-        <f>(G1656/G1604)-1</f>
-        <v>-0.23076923076923073</v>
-      </c>
-      <c r="H1667" s="20"/>
-      <c r="I1667" s="20">
-        <f>(I1656/I1604)-1</f>
-        <v>-0.31914893617021278</v>
-      </c>
+      <c r="B1667" s="1"/>
+      <c r="C1667" s="1"/>
+      <c r="D1667" s="1"/>
       <c r="P1667" s="2"/>
       <c r="Q1667" s="2"/>
       <c r="R1667" s="2"/>
     </row>
     <row r="1668" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1668" s="16" t="s">
-        <v>1626</v>
-      </c>
-      <c r="E1668" s="17">
-        <f>(E1656/F1656)-1</f>
-        <v>-0.11111111111111116</v>
-      </c>
-      <c r="G1668" s="17">
-        <f>(G1656/H1656)-1</f>
-        <v>-0.13978494623655913</v>
-      </c>
-      <c r="I1668" s="17">
-        <f>(I1656/J1656)-1</f>
-        <v>-0.23353293413173648</v>
+      <c r="B1668" s="1"/>
+      <c r="C1668" s="1"/>
+      <c r="D1668" s="1"/>
+      <c r="E1668" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1668" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1668" s="3" t="s">
+        <v>3</v>
       </c>
       <c r="P1668" s="2"/>
       <c r="Q1668" s="2"/>
       <c r="R1668" s="2"/>
     </row>
     <row r="1669" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1669" s="14"/>
-      <c r="C1669" s="1"/>
-      <c r="D1669" s="1"/>
+      <c r="E1669" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1669" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1669" s="39" t="s">
+        <v>1623</v>
+      </c>
+      <c r="L1669" s="1" t="s">
+        <v>1624</v>
+      </c>
       <c r="P1669" s="2"/>
       <c r="Q1669" s="2"/>
       <c r="R1669" s="2"/>
     </row>
     <row r="1670" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1670" s="14"/>
-      <c r="C1670" s="1"/>
-      <c r="D1670" s="1"/>
+      <c r="A1670" s="16" t="s">
+        <v>1625</v>
+      </c>
+      <c r="E1670" s="20">
+        <f>(E1657/E1605)-1</f>
+        <v>-0.14814814814814814</v>
+      </c>
+      <c r="F1670" s="20"/>
+      <c r="G1670" s="20">
+        <f>(G1657/G1605)-1</f>
+        <v>-0.26666666666666672</v>
+      </c>
+      <c r="H1670" s="20"/>
+      <c r="I1670" s="20">
+        <f>(I1657/I1605)-1</f>
+        <v>-0.10909090909090913</v>
+      </c>
       <c r="P1670" s="2"/>
       <c r="Q1670" s="2"/>
       <c r="R1670" s="2"/>
     </row>
     <row r="1671" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1671" s="14"/>
-      <c r="C1671" s="1"/>
-      <c r="D1671" s="1"/>
+      <c r="A1671" s="16" t="s">
+        <v>1626</v>
+      </c>
+      <c r="E1671" s="17">
+        <f>(E1657/F1657)-1</f>
+        <v>-0.14814814814814814</v>
+      </c>
+      <c r="G1671" s="17">
+        <f>(G1657/H1657)-1</f>
+        <v>-9.2783505154639179E-2</v>
+      </c>
+      <c r="I1671" s="17">
+        <f>(I1657/J1657)-1</f>
+        <v>2.6178010471204161E-2</v>
+      </c>
       <c r="P1671" s="2"/>
       <c r="Q1671" s="2"/>
       <c r="R1671" s="2"/>
@@ -83873,179 +83919,203 @@
     </row>
     <row r="1745" spans="1:24" x14ac:dyDescent="0.25">
       <c r="B1745" s="14"/>
-      <c r="C1745" s="14"/>
-      <c r="D1745" s="14"/>
+      <c r="C1745" s="1"/>
+      <c r="D1745" s="1"/>
       <c r="P1745" s="2"/>
       <c r="Q1745" s="2"/>
       <c r="R1745" s="2"/>
     </row>
     <row r="1746" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1746" s="14" t="s">
-        <v>1618</v>
-      </c>
-      <c r="C1746" s="14"/>
-      <c r="D1746" s="14"/>
-      <c r="E1746" s="26">
-        <f>AVERAGE(E1047:E1099)</f>
-        <v>42.490566037735846</v>
-      </c>
-      <c r="F1746" s="26"/>
-      <c r="G1746" s="26">
-        <f>AVERAGE(G1047:G1099)</f>
-        <v>37.641509433962263</v>
-      </c>
-      <c r="H1746" s="26"/>
-      <c r="I1746" s="26">
-        <f>AVERAGE(I1047:I1099)</f>
-        <v>56.320754716981135</v>
-      </c>
-      <c r="M1746" s="26"/>
+      <c r="B1746" s="14"/>
+      <c r="C1746" s="1"/>
+      <c r="D1746" s="1"/>
       <c r="P1746" s="2"/>
       <c r="Q1746" s="2"/>
       <c r="R1746" s="2"/>
     </row>
     <row r="1747" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1747" s="25" t="s">
-        <v>1619</v>
-      </c>
-      <c r="C1747" s="25"/>
-      <c r="D1747" s="25"/>
-      <c r="E1747" s="1" t="s">
-        <v>1620</v>
-      </c>
-      <c r="G1747" s="1" t="s">
-        <v>1621</v>
-      </c>
-      <c r="I1747" s="1" t="s">
-        <v>1622</v>
-      </c>
+      <c r="B1747" s="14"/>
+      <c r="C1747" s="1"/>
+      <c r="D1747" s="1"/>
       <c r="P1747" s="2"/>
       <c r="Q1747" s="2"/>
       <c r="R1747" s="2"/>
     </row>
     <row r="1748" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1748" s="1"/>
-      <c r="C1748" s="1"/>
-      <c r="D1748" s="1"/>
+      <c r="B1748" s="14"/>
+      <c r="C1748" s="14"/>
+      <c r="D1748" s="14"/>
       <c r="P1748" s="2"/>
       <c r="Q1748" s="2"/>
       <c r="R1748" s="2"/>
     </row>
     <row r="1749" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1749" s="1"/>
-      <c r="C1749" s="1"/>
-      <c r="D1749" s="1"/>
-      <c r="E1749" s="3" t="s">
+      <c r="B1749" s="14" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C1749" s="14"/>
+      <c r="D1749" s="14"/>
+      <c r="E1749" s="26">
+        <f>AVERAGE(E1047:E1099)</f>
+        <v>42.490566037735846</v>
+      </c>
+      <c r="F1749" s="26"/>
+      <c r="G1749" s="26">
+        <f>AVERAGE(G1047:G1099)</f>
+        <v>37.641509433962263</v>
+      </c>
+      <c r="H1749" s="26"/>
+      <c r="I1749" s="26">
+        <f>AVERAGE(I1047:I1099)</f>
+        <v>56.320754716981135</v>
+      </c>
+      <c r="M1749" s="26"/>
+      <c r="P1749" s="2"/>
+      <c r="Q1749" s="2"/>
+      <c r="R1749" s="2"/>
+    </row>
+    <row r="1750" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B1750" s="25" t="s">
+        <v>1619</v>
+      </c>
+      <c r="C1750" s="25"/>
+      <c r="D1750" s="25"/>
+      <c r="E1750" s="1" t="s">
+        <v>1620</v>
+      </c>
+      <c r="G1750" s="1" t="s">
+        <v>1621</v>
+      </c>
+      <c r="I1750" s="1" t="s">
+        <v>1622</v>
+      </c>
+      <c r="P1750" s="2"/>
+      <c r="Q1750" s="2"/>
+      <c r="R1750" s="2"/>
+    </row>
+    <row r="1751" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B1751" s="1"/>
+      <c r="C1751" s="1"/>
+      <c r="D1751" s="1"/>
+      <c r="P1751" s="2"/>
+      <c r="Q1751" s="2"/>
+      <c r="R1751" s="2"/>
+    </row>
+    <row r="1752" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B1752" s="1"/>
+      <c r="C1752" s="1"/>
+      <c r="D1752" s="1"/>
+      <c r="E1752" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1749" s="3" t="s">
+      <c r="G1752" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I1749" s="3" t="s">
+      <c r="I1752" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="Q1749" s="1" t="s">
+      <c r="Q1752" s="1" t="s">
         <v>1624</v>
       </c>
     </row>
-    <row r="1750" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="E1750" s="3" t="s">
+    <row r="1753" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="E1753" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G1750" s="3" t="s">
+      <c r="G1753" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I1750" s="39" t="s">
+      <c r="I1753" s="39" t="s">
         <v>1623</v>
       </c>
     </row>
-    <row r="1751" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1751" s="16" t="s">
+    <row r="1754" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1754" s="16" t="s">
         <v>1625</v>
       </c>
-      <c r="E1751" s="20">
+      <c r="E1754" s="20">
         <f>(E1441/E1389)-1</f>
         <v>-0.51724137931034475</v>
       </c>
-      <c r="F1751" s="20"/>
-      <c r="G1751" s="20">
+      <c r="F1754" s="20"/>
+      <c r="G1754" s="20">
         <f>(G1441/G1389)-1</f>
         <v>0</v>
       </c>
-      <c r="H1751" s="20"/>
-      <c r="I1751" s="20">
+      <c r="H1754" s="20"/>
+      <c r="I1754" s="20">
         <f>(I1441/I1389)-1</f>
         <v>0.1020408163265305</v>
       </c>
-      <c r="M1751" s="4"/>
-      <c r="N1751" s="17"/>
-      <c r="O1751" s="4"/>
-    </row>
-    <row r="1752" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1752" s="16" t="s">
+      <c r="M1754" s="4"/>
+      <c r="N1754" s="17"/>
+      <c r="O1754" s="4"/>
+    </row>
+    <row r="1755" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1755" s="16" t="s">
         <v>1626</v>
       </c>
-      <c r="E1752" s="17">
+      <c r="E1755" s="17">
         <f>(E1441/F1441)-1</f>
         <v>-0.55555555555555558</v>
       </c>
-      <c r="G1752" s="17">
+      <c r="G1755" s="17">
         <f>(G1441/H1441)-1</f>
         <v>-0.1333333333333333</v>
       </c>
-      <c r="I1752" s="17">
+      <c r="I1755" s="17">
         <f>(I1441/J1441)-1</f>
         <v>0.17391304347826098</v>
       </c>
-      <c r="P1752" s="26"/>
-      <c r="Q1752" s="26"/>
-      <c r="R1752" s="26"/>
-      <c r="S1752" s="26"/>
-    </row>
-    <row r="1753" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1753" s="16"/>
-    </row>
-    <row r="1754" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1754" s="16"/>
-    </row>
-    <row r="1755" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1755" s="16"/>
-      <c r="N1755" s="17"/>
-      <c r="O1755" s="24"/>
+      <c r="P1755" s="26"/>
+      <c r="Q1755" s="26"/>
+      <c r="R1755" s="26"/>
+      <c r="S1755" s="26"/>
     </row>
     <row r="1756" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1756" s="16"/>
-      <c r="P1756" s="4"/>
-      <c r="Q1756" s="4"/>
-      <c r="R1756" s="4"/>
-      <c r="S1756" s="4"/>
-      <c r="V1756" s="4"/>
-      <c r="W1756" s="4"/>
-      <c r="X1756" s="4"/>
+    </row>
+    <row r="1757" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1757" s="16"/>
     </row>
     <row r="1758" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="M1758" s="17"/>
+      <c r="A1758" s="16"/>
+      <c r="N1758" s="17"/>
+      <c r="O1758" s="24"/>
     </row>
     <row r="1759" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="M1759" s="17"/>
-    </row>
-    <row r="1764" spans="6:17" x14ac:dyDescent="0.25">
-      <c r="N1764" s="21"/>
-      <c r="O1764" s="21"/>
-      <c r="P1764" s="21"/>
-      <c r="Q1764" s="21"/>
-    </row>
-    <row r="1766" spans="6:17" x14ac:dyDescent="0.25">
-      <c r="F1766" s="2"/>
-    </row>
-    <row r="1815" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I1815" s="2"/>
-    </row>
-    <row r="1826" spans="16:19" x14ac:dyDescent="0.25">
-      <c r="P1826" s="4"/>
-      <c r="Q1826" s="4"/>
-      <c r="R1826" s="4"/>
-      <c r="S1826" s="4"/>
+      <c r="A1759" s="16"/>
+      <c r="P1759" s="4"/>
+      <c r="Q1759" s="4"/>
+      <c r="R1759" s="4"/>
+      <c r="S1759" s="4"/>
+      <c r="V1759" s="4"/>
+      <c r="W1759" s="4"/>
+      <c r="X1759" s="4"/>
+    </row>
+    <row r="1761" spans="6:17" x14ac:dyDescent="0.25">
+      <c r="M1761" s="17"/>
+    </row>
+    <row r="1762" spans="6:17" x14ac:dyDescent="0.25">
+      <c r="M1762" s="17"/>
+    </row>
+    <row r="1767" spans="6:17" x14ac:dyDescent="0.25">
+      <c r="N1767" s="21"/>
+      <c r="O1767" s="21"/>
+      <c r="P1767" s="21"/>
+      <c r="Q1767" s="21"/>
+    </row>
+    <row r="1769" spans="6:17" x14ac:dyDescent="0.25">
+      <c r="F1769" s="2"/>
+    </row>
+    <row r="1818" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I1818" s="2"/>
+    </row>
+    <row r="1829" spans="16:19" x14ac:dyDescent="0.25">
+      <c r="P1829" s="4"/>
+      <c r="Q1829" s="4"/>
+      <c r="R1829" s="4"/>
+      <c r="S1829" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A927:A932" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -84060,7 +84130,7 @@
   <pageSetup orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <ignoredErrors>
-    <ignoredError sqref="E1746:I1746 E1662:I1662" formulaRange="1"/>
+    <ignoredError sqref="E1749:I1749 E1665:I1665" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -84098,99 +84168,99 @@
       <c r="G2" s="15"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="60" t="s">
+      <c r="B3" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="60" t="s">
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="61" t="s">
         <v>1629</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="15"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="63"/>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="61"/>
+      <c r="A4" s="64"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="62"/>
       <c r="F4" s="15"/>
       <c r="G4" s="15"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="63"/>
-      <c r="B5" s="60" t="s">
+      <c r="A5" s="64"/>
+      <c r="B5" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="60" t="s">
+      <c r="C5" s="61" t="s">
         <v>1630</v>
       </c>
-      <c r="D5" s="60" t="s">
+      <c r="D5" s="61" t="s">
         <v>1631</v>
       </c>
-      <c r="E5" s="60" t="s">
+      <c r="E5" s="61" t="s">
         <v>1</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="64"/>
-      <c r="B6" s="61"/>
-      <c r="C6" s="61"/>
-      <c r="D6" s="61"/>
-      <c r="E6" s="61"/>
+      <c r="A6" s="65"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="30">
+        <f>Data!A1657</f>
+        <v>46275</v>
+      </c>
+      <c r="B7" s="27">
+        <f>Data!E1657</f>
+        <v>23</v>
+      </c>
+      <c r="C7" s="27">
+        <f>Data!G1657</f>
+        <v>22</v>
+      </c>
+      <c r="D7" s="27">
+        <f>Data!I1657</f>
+        <v>49</v>
+      </c>
+      <c r="E7" s="54">
+        <f>Data!M1657</f>
+        <v>11</v>
+      </c>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="30">
         <f>Data!A1656</f>
         <v>46268</v>
       </c>
-      <c r="B7" s="27">
+      <c r="B8" s="27">
         <f>Data!E1656</f>
         <v>22</v>
       </c>
-      <c r="C7" s="27">
+      <c r="C8" s="27">
         <f>Data!G1656</f>
         <v>20</v>
       </c>
-      <c r="D7" s="27">
+      <c r="D8" s="27">
         <f>Data!I1656</f>
         <v>32</v>
       </c>
-      <c r="E7" s="54">
+      <c r="E8" s="54">
         <f>Data!M1656</f>
         <v>12</v>
-      </c>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="30">
-        <f>Data!A1655</f>
-        <v>46261</v>
-      </c>
-      <c r="B8" s="27">
-        <f>Data!E1655</f>
-        <v>10</v>
-      </c>
-      <c r="C8" s="27">
-        <f>Data!G1655</f>
-        <v>18</v>
-      </c>
-      <c r="D8" s="27">
-        <f>Data!I1655</f>
-        <v>29</v>
-      </c>
-      <c r="E8" s="54">
-        <f>Data!M1655</f>
-        <v>13</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
@@ -84499,7 +84569,9 @@
       <c r="L11" s="15"/>
       <c r="M11" s="15"/>
       <c r="N11" s="15"/>
-      <c r="O11" s="15"/>
+      <c r="O11" s="58" t="s">
+        <v>1691</v>
+      </c>
       <c r="P11" s="15"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
@@ -85053,7 +85125,7 @@
   <sheetData>
     <row r="5" spans="4:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D5" s="43" t="s">
-        <v>1691</v>
+        <v>1693</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>2</v>
@@ -85067,10 +85139,10 @@
         <v>1635</v>
       </c>
       <c r="E6" s="50">
-        <v>-0.23100000000000001</v>
+        <v>-0.26700000000000002</v>
       </c>
       <c r="F6" s="51">
-        <v>-0.31900000000000001</v>
+        <v>-0.109</v>
       </c>
     </row>
     <row r="7" spans="4:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -85078,10 +85150,10 @@
         <v>1636</v>
       </c>
       <c r="E7" s="57">
-        <v>-0.14000000000000001</v>
+        <v>-9.2999999999999999E-2</v>
       </c>
       <c r="F7" s="52">
-        <v>-0.23400000000000001</v>
+        <v>2.5999999999999999E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data: Intermodal W40/W41, Banchero W41, Alibra 10-14 re-parsed; leaks repaired; feeds caught up
- Intermodal W40/W41 MDs + sidecars (Nace); W41 tanker spot rebuilt from the PDF text
  layer (Nace had shifted every label one row). Rows appended to the 16 Intermodal
  series CSVs (no existing rows changed); every appended number is on the text layer.
- Banchero W41 and Alibra 10-14 dry/wet re-parsed; Alibra trends checked against images.
- Nace prompt-leak lines repaired: Stopford p251, RIO 6-K 2026-03-02 and 2026-10-01.
- Root-level duplicate MDs removed (Xclusiv x2, ISM, stale Banchero W40 with dropped
  chart_series); SSY root MDs moved into 2026/.
- USDA FAS/inspections/queues and Argentina grain caught up (source revisions included).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/commodities/GTRTable19_Figure19.xlsx
+++ b/data/commodities/GTRTable19_Figure19.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdagcc.sharepoint.com/sites/MRP-AMS-TED/Shared Documents/GTR/WebZip Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="396" documentId="8_{5DC5C50C-B9D1-43B8-8139-6A342E8B45D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DCD68E3-E672-4CA4-BDA5-99076DE74552}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{D5E42450-2855-4A44-AD8D-155DB7860793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB901717-DFBD-4A8B-B503-A5766A807741}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4252" uniqueCount="1694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4268" uniqueCount="1698">
   <si>
     <t>Gulf</t>
   </si>
@@ -5124,7 +5124,19 @@
     <t>09/10/2026</t>
   </si>
   <si>
-    <t>Week ending 09/10/26, number of vessels</t>
+    <t>09/17/2026</t>
+  </si>
+  <si>
+    <t>09/24/2026</t>
+  </si>
+  <si>
+    <t>10/01/2026</t>
+  </si>
+  <si>
+    <t>10/08/2026</t>
+  </si>
+  <si>
+    <t>Week ending 10/08/26, number of vessels</t>
   </si>
 </sst>
 </file>
@@ -5689,215 +5701,215 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$B$1625:$B$1657</c:f>
+              <c:f>Data!$B$1629:$B$1661</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>01/29/2026</c:v>
+                  <c:v>02/26/2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>02/05/2026</c:v>
+                  <c:v>03/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>02/12/2026</c:v>
+                  <c:v>03/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>02/19/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>02/26/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>03/05/2026</c:v>
+                  <c:v>04/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>03/12/2026</c:v>
+                  <c:v>04/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>04/02/2026</c:v>
+                  <c:v>04/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>04/09/2026</c:v>
+                  <c:v>05/07/2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>04/16/2026</c:v>
+                  <c:v>05/14/2026</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>04/23/2026</c:v>
+                  <c:v>05/21/2026</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>04/30/2026</c:v>
+                  <c:v>05/28/2026</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>05/07/2026</c:v>
+                  <c:v>06/04/2026</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>05/14/2026</c:v>
+                  <c:v>06/11/2026</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>05/21/2026</c:v>
+                  <c:v>06/18/2026</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>05/28/2026</c:v>
+                  <c:v>06/25/2026</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>06/04/2026</c:v>
+                  <c:v>07/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>06/11/2026</c:v>
+                  <c:v>07/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>06/18/2026</c:v>
+                  <c:v>07/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>06/25/2026</c:v>
+                  <c:v>07/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>07/02/2026</c:v>
+                  <c:v>07/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>07/09/2026</c:v>
+                  <c:v>08/06/2026</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>07/16/2026</c:v>
+                  <c:v>08/13/2026</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>07/23/2026</c:v>
+                  <c:v>08/20/2026</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>07/30/2026</c:v>
+                  <c:v>08/27/2026</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>08/06/2026</c:v>
+                  <c:v>09/03/2026</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>08/13/2026</c:v>
+                  <c:v>09/10/2026</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>08/20/2026</c:v>
+                  <c:v>09/17/2026</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>08/27/2026</c:v>
+                  <c:v>09/24/2026</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>09/03/2026</c:v>
+                  <c:v>10/01/2026</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>09/10/2026</c:v>
+                  <c:v>10/08/2026</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$G$1625:$G$1657</c:f>
+              <c:f>Data!$G$1629:$G$1661</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>31</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>34</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>34</c:v>
-                </c:pt>
                 <c:pt idx="6">
-                  <c:v>32</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>40</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>33</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="19">
                   <c:v>30</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="20">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="22">
                   <c:v>27</c:v>
                 </c:pt>
-                <c:pt idx="12">
-                  <c:v>26</c:v>
+                <c:pt idx="23">
+                  <c:v>33</c:v>
                 </c:pt>
-                <c:pt idx="13">
+                <c:pt idx="24">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="14">
+                <c:pt idx="25">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="30">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="15">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>36</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>32</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>33</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>29</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>18</c:v>
-                </c:pt>
                 <c:pt idx="31">
-                  <c:v>20</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>22</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5927,215 +5939,215 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$B$1625:$B$1657</c:f>
+              <c:f>Data!$B$1629:$B$1661</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>01/29/2026</c:v>
+                  <c:v>02/26/2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>02/05/2026</c:v>
+                  <c:v>03/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>02/12/2026</c:v>
+                  <c:v>03/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>02/19/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>02/26/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>03/05/2026</c:v>
+                  <c:v>04/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>03/12/2026</c:v>
+                  <c:v>04/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>04/02/2026</c:v>
+                  <c:v>04/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>04/09/2026</c:v>
+                  <c:v>05/07/2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>04/16/2026</c:v>
+                  <c:v>05/14/2026</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>04/23/2026</c:v>
+                  <c:v>05/21/2026</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>04/30/2026</c:v>
+                  <c:v>05/28/2026</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>05/07/2026</c:v>
+                  <c:v>06/04/2026</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>05/14/2026</c:v>
+                  <c:v>06/11/2026</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>05/21/2026</c:v>
+                  <c:v>06/18/2026</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>05/28/2026</c:v>
+                  <c:v>06/25/2026</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>06/04/2026</c:v>
+                  <c:v>07/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>06/11/2026</c:v>
+                  <c:v>07/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>06/18/2026</c:v>
+                  <c:v>07/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>06/25/2026</c:v>
+                  <c:v>07/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>07/02/2026</c:v>
+                  <c:v>07/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>07/09/2026</c:v>
+                  <c:v>08/06/2026</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>07/16/2026</c:v>
+                  <c:v>08/13/2026</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>07/23/2026</c:v>
+                  <c:v>08/20/2026</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>07/30/2026</c:v>
+                  <c:v>08/27/2026</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>08/06/2026</c:v>
+                  <c:v>09/03/2026</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>08/13/2026</c:v>
+                  <c:v>09/10/2026</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>08/20/2026</c:v>
+                  <c:v>09/17/2026</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>08/27/2026</c:v>
+                  <c:v>09/24/2026</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>09/03/2026</c:v>
+                  <c:v>10/01/2026</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>09/10/2026</c:v>
+                  <c:v>10/08/2026</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$I$1625:$I$1657</c:f>
+              <c:f>Data!$I$1629:$I$1661</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>61</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>50</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>40</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>37</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>48</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>58</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>58</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>36</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>41</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>33</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>40</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>42</c:v>
+                  <c:v>38</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>48</c:v>
+                  <c:v>29</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>37</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>38</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="18">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="26">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="19">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>37</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>42</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>41</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>28</c:v>
-                </c:pt>
                 <c:pt idx="27">
-                  <c:v>30</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>31</c:v>
+                  <c:v>49</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>30</c:v>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>29</c:v>
+                  <c:v>47</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>32</c:v>
+                  <c:v>44</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>49</c:v>
+                  <c:v>46</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6192,215 +6204,215 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$B$1625:$B$1657</c:f>
+              <c:f>Data!$B$1629:$B$1661</c:f>
               <c:strCache>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
-                  <c:v>01/29/2026</c:v>
+                  <c:v>02/26/2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>02/05/2026</c:v>
+                  <c:v>03/05/2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>02/12/2026</c:v>
+                  <c:v>03/12/2026</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>02/19/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>02/26/2026</c:v>
+                  <c:v>03/19/2026</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>03/05/2026</c:v>
+                  <c:v>04/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>03/12/2026</c:v>
+                  <c:v>04/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>03/19/2026</c:v>
+                  <c:v>04/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>04/02/2026</c:v>
+                  <c:v>04/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>04/09/2026</c:v>
+                  <c:v>05/07/2026</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>04/16/2026</c:v>
+                  <c:v>05/14/2026</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>04/23/2026</c:v>
+                  <c:v>05/21/2026</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>04/30/2026</c:v>
+                  <c:v>05/28/2026</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>05/07/2026</c:v>
+                  <c:v>06/04/2026</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>05/14/2026</c:v>
+                  <c:v>06/11/2026</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>05/21/2026</c:v>
+                  <c:v>06/18/2026</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>05/28/2026</c:v>
+                  <c:v>06/25/2026</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>06/04/2026</c:v>
+                  <c:v>07/02/2026</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>06/11/2026</c:v>
+                  <c:v>07/09/2026</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>06/18/2026</c:v>
+                  <c:v>07/16/2026</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>06/25/2026</c:v>
+                  <c:v>07/23/2026</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>07/02/2026</c:v>
+                  <c:v>07/30/2026</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>07/09/2026</c:v>
+                  <c:v>08/06/2026</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>07/16/2026</c:v>
+                  <c:v>08/13/2026</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>07/23/2026</c:v>
+                  <c:v>08/20/2026</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>07/30/2026</c:v>
+                  <c:v>08/27/2026</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>08/06/2026</c:v>
+                  <c:v>09/03/2026</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>08/13/2026</c:v>
+                  <c:v>09/10/2026</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>08/20/2026</c:v>
+                  <c:v>09/17/2026</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>08/27/2026</c:v>
+                  <c:v>09/24/2026</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>09/03/2026</c:v>
+                  <c:v>10/01/2026</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>09/10/2026</c:v>
+                  <c:v>10/08/2026</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$H$1625:$H$1657</c:f>
+              <c:f>Data!$H$1629:$H$1661</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="33"/>
                 <c:pt idx="0">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>29</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>31.25</c:v>
-                </c:pt>
                 <c:pt idx="2">
-                  <c:v>32.25</c:v>
+                  <c:v>31.75</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>27.25</c:v>
+                  <c:v>31.25</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>29</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>31.75</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>31.25</c:v>
-                </c:pt>
                 <c:pt idx="8">
-                  <c:v>31</c:v>
+                  <c:v>29.25</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>30</c:v>
+                  <c:v>26.75</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>24.75</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>22.75</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>23.5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>26.5</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>25.75</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>20.75</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>20.25</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>20.75</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>22.25</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>23.25</c:v>
+                </c:pt>
+                <c:pt idx="22">
                   <c:v>28</c:v>
                 </c:pt>
-                <c:pt idx="11">
-                  <c:v>31.75</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>29.25</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>26.75</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>24.75</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>22.75</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>23.5</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>26.5</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>25.75</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>20.75</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>20.25</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>20.75</c:v>
-                </c:pt>
                 <c:pt idx="23">
-                  <c:v>22.25</c:v>
+                  <c:v>22.5</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>22</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="25">
+                  <c:v>22.5</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="27">
                   <c:v>23.25</c:v>
                 </c:pt>
-                <c:pt idx="26">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>22.5</c:v>
-                </c:pt>
                 <c:pt idx="28">
-                  <c:v>19</c:v>
+                  <c:v>24.25</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>22.5</c:v>
+                  <c:v>27.25</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>26</c:v>
+                  <c:v>27.75</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>23.25</c:v>
+                  <c:v>29.5</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>24.25</c:v>
+                  <c:v>27.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6972,7 +6984,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:X1829"/>
+  <dimension ref="A1:X1833"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="12" bestFit="1" customWidth="1"/>
@@ -79814,14 +79826,14 @@
         <v>26</v>
       </c>
       <c r="H1598" s="1">
-        <f t="shared" ref="H1598:H1657" si="87">AVERAGE(G1546,G1494,G1442,G1390)</f>
+        <f t="shared" ref="H1598:H1661" si="87">AVERAGE(G1546,G1494,G1442,G1390)</f>
         <v>25.75</v>
       </c>
       <c r="I1598" s="1">
         <v>37</v>
       </c>
       <c r="J1598" s="1">
-        <f t="shared" ref="J1598:J1657" si="88">AVERAGE(I1546,I1494,I1442,I1390)</f>
+        <f t="shared" ref="J1598:J1661" si="88">AVERAGE(I1546,I1494,I1442,I1390)</f>
         <v>39.75</v>
       </c>
       <c r="K1598" s="1">
@@ -82327,7 +82339,7 @@
         <v>20</v>
       </c>
       <c r="F1643" s="1">
-        <f t="shared" ref="F1643:F1657" si="89">AVERAGE(E1591,E1539,E1487,E1435)</f>
+        <f t="shared" ref="F1643:F1661" si="89">AVERAGE(E1591,E1539,E1487,E1435)</f>
         <v>19</v>
       </c>
       <c r="G1643" s="1">
@@ -83151,36 +83163,228 @@
       </c>
     </row>
     <row r="1658" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1658" s="48"/>
-      <c r="C1658" s="1"/>
-      <c r="D1658" s="1"/>
-      <c r="P1658" s="2"/>
-      <c r="Q1658" s="2"/>
-      <c r="R1658" s="2"/>
+      <c r="A1658" s="12">
+        <v>46282</v>
+      </c>
+      <c r="B1658" s="48" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C1658" s="1">
+        <v>9</v>
+      </c>
+      <c r="D1658" s="1">
+        <v>12</v>
+      </c>
+      <c r="E1658" s="1">
+        <v>21</v>
+      </c>
+      <c r="F1658" s="1">
+        <f t="shared" si="89"/>
+        <v>30.5</v>
+      </c>
+      <c r="G1658" s="1">
+        <v>28</v>
+      </c>
+      <c r="H1658" s="1">
+        <f t="shared" si="87"/>
+        <v>27.25</v>
+      </c>
+      <c r="I1658" s="1">
+        <v>51</v>
+      </c>
+      <c r="J1658" s="1">
+        <f t="shared" si="88"/>
+        <v>43.25</v>
+      </c>
+      <c r="K1658" s="1">
+        <v>3</v>
+      </c>
+      <c r="L1658" s="1">
+        <v>11</v>
+      </c>
+      <c r="M1658" s="1">
+        <v>14</v>
+      </c>
+      <c r="P1658" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="Q1658" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="R1658" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="S1658" s="1">
+        <v>37</v>
+      </c>
     </row>
     <row r="1659" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1659" s="48"/>
-      <c r="C1659" s="1"/>
-      <c r="D1659" s="1"/>
-      <c r="P1659" s="2"/>
-      <c r="Q1659" s="2"/>
-      <c r="R1659" s="2"/>
+      <c r="A1659" s="12">
+        <v>46289</v>
+      </c>
+      <c r="B1659" s="48" t="s">
+        <v>1694</v>
+      </c>
+      <c r="C1659" s="1">
+        <v>8</v>
+      </c>
+      <c r="D1659" s="1">
+        <v>17</v>
+      </c>
+      <c r="E1659" s="1">
+        <v>25</v>
+      </c>
+      <c r="F1659" s="1">
+        <f t="shared" si="89"/>
+        <v>32</v>
+      </c>
+      <c r="G1659" s="1">
+        <v>29</v>
+      </c>
+      <c r="H1659" s="1">
+        <f t="shared" si="87"/>
+        <v>27.75</v>
+      </c>
+      <c r="I1659" s="1">
+        <v>47</v>
+      </c>
+      <c r="J1659" s="1">
+        <f t="shared" si="88"/>
+        <v>45.25</v>
+      </c>
+      <c r="K1659" s="1">
+        <v>5</v>
+      </c>
+      <c r="L1659" s="1">
+        <v>6</v>
+      </c>
+      <c r="M1659" s="1">
+        <v>11</v>
+      </c>
+      <c r="P1659" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="Q1659" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="R1659" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="S1659" s="1">
+        <v>38</v>
+      </c>
     </row>
     <row r="1660" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1660" s="48"/>
-      <c r="C1660" s="1"/>
-      <c r="D1660" s="1"/>
-      <c r="P1660" s="2"/>
-      <c r="Q1660" s="2"/>
-      <c r="R1660" s="2"/>
+      <c r="A1660" s="12">
+        <v>46296</v>
+      </c>
+      <c r="B1660" s="48" t="s">
+        <v>1695</v>
+      </c>
+      <c r="C1660" s="1">
+        <v>10</v>
+      </c>
+      <c r="D1660" s="1">
+        <v>13</v>
+      </c>
+      <c r="E1660" s="1">
+        <v>23</v>
+      </c>
+      <c r="F1660" s="1">
+        <f t="shared" si="89"/>
+        <v>33.75</v>
+      </c>
+      <c r="G1660" s="1">
+        <v>39</v>
+      </c>
+      <c r="H1660" s="1">
+        <f t="shared" si="87"/>
+        <v>29.5</v>
+      </c>
+      <c r="I1660" s="1">
+        <v>44</v>
+      </c>
+      <c r="J1660" s="1">
+        <f t="shared" si="88"/>
+        <v>48.5</v>
+      </c>
+      <c r="K1660" s="1">
+        <v>4</v>
+      </c>
+      <c r="L1660" s="1">
+        <v>12</v>
+      </c>
+      <c r="M1660" s="1">
+        <v>16</v>
+      </c>
+      <c r="P1660" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="Q1660" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="R1660" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="S1660" s="1">
+        <v>39</v>
+      </c>
     </row>
     <row r="1661" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1661" s="48"/>
-      <c r="C1661" s="1"/>
-      <c r="D1661" s="1"/>
-      <c r="P1661" s="2"/>
-      <c r="Q1661" s="2"/>
-      <c r="R1661" s="2"/>
+      <c r="A1661" s="12">
+        <v>46303</v>
+      </c>
+      <c r="B1661" s="48" t="s">
+        <v>1696</v>
+      </c>
+      <c r="C1661" s="1">
+        <v>9</v>
+      </c>
+      <c r="D1661" s="1">
+        <v>18</v>
+      </c>
+      <c r="E1661" s="1">
+        <v>27</v>
+      </c>
+      <c r="F1661" s="1">
+        <f t="shared" si="89"/>
+        <v>32.5</v>
+      </c>
+      <c r="G1661" s="1">
+        <v>28</v>
+      </c>
+      <c r="H1661" s="1">
+        <f t="shared" si="87"/>
+        <v>27.25</v>
+      </c>
+      <c r="I1661" s="1">
+        <v>46</v>
+      </c>
+      <c r="J1661" s="1">
+        <f t="shared" si="88"/>
+        <v>49.75</v>
+      </c>
+      <c r="K1661" s="1">
+        <v>5</v>
+      </c>
+      <c r="L1661" s="1">
+        <v>12</v>
+      </c>
+      <c r="M1661" s="1">
+        <v>17</v>
+      </c>
+      <c r="P1661" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="Q1661" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="R1661" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="S1661" s="1">
+        <v>40</v>
+      </c>
     </row>
     <row r="1662" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1662" s="48"/>
@@ -83191,7 +83395,7 @@
       <c r="R1662" s="2"/>
     </row>
     <row r="1663" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1663" s="14"/>
+      <c r="B1663" s="48"/>
       <c r="C1663" s="1"/>
       <c r="D1663" s="1"/>
       <c r="P1663" s="2"/>
@@ -83199,7 +83403,7 @@
       <c r="R1663" s="2"/>
     </row>
     <row r="1664" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B1664" s="14"/>
+      <c r="B1664" s="48"/>
       <c r="C1664" s="1"/>
       <c r="D1664" s="1"/>
       <c r="P1664" s="2"/>
@@ -83207,50 +83411,23 @@
       <c r="R1664" s="2"/>
     </row>
     <row r="1665" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1665" s="14" t="s">
-        <v>1618</v>
-      </c>
-      <c r="C1665" s="14"/>
-      <c r="D1665" s="14"/>
-      <c r="E1665" s="26">
-        <f>AVERAGE(E1050:E1102)</f>
-        <v>43.075471698113205</v>
-      </c>
-      <c r="F1665" s="26"/>
-      <c r="G1665" s="26">
-        <f>AVERAGE(G1050:G1102)</f>
-        <v>37.433962264150942</v>
-      </c>
-      <c r="H1665" s="26"/>
-      <c r="I1665" s="26">
-        <f>AVERAGE(I1050:I1102)</f>
-        <v>56.113207547169814</v>
-      </c>
+      <c r="B1665" s="48"/>
+      <c r="C1665" s="1"/>
+      <c r="D1665" s="1"/>
       <c r="P1665" s="2"/>
       <c r="Q1665" s="2"/>
       <c r="R1665" s="2"/>
     </row>
     <row r="1666" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1666" s="25" t="s">
-        <v>1619</v>
-      </c>
-      <c r="C1666" s="25"/>
-      <c r="D1666" s="25"/>
-      <c r="E1666" s="1" t="s">
-        <v>1620</v>
-      </c>
-      <c r="G1666" s="1" t="s">
-        <v>1621</v>
-      </c>
-      <c r="I1666" s="1" t="s">
-        <v>1622</v>
-      </c>
+      <c r="B1666" s="48"/>
+      <c r="C1666" s="1"/>
+      <c r="D1666" s="1"/>
       <c r="P1666" s="2"/>
       <c r="Q1666" s="2"/>
       <c r="R1666" s="2"/>
     </row>
     <row r="1667" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1667" s="1"/>
+      <c r="B1667" s="14"/>
       <c r="C1667" s="1"/>
       <c r="D1667" s="1"/>
       <c r="P1667" s="2"/>
@@ -83258,109 +83435,136 @@
       <c r="R1667" s="2"/>
     </row>
     <row r="1668" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1668" s="1"/>
+      <c r="B1668" s="14"/>
       <c r="C1668" s="1"/>
       <c r="D1668" s="1"/>
-      <c r="E1668" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1668" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1668" s="3" t="s">
-        <v>3</v>
-      </c>
       <c r="P1668" s="2"/>
       <c r="Q1668" s="2"/>
       <c r="R1668" s="2"/>
     </row>
     <row r="1669" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="E1669" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1669" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1669" s="39" t="s">
-        <v>1623</v>
-      </c>
-      <c r="L1669" s="1" t="s">
-        <v>1624</v>
+      <c r="B1669" s="14" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C1669" s="14"/>
+      <c r="D1669" s="14"/>
+      <c r="E1669" s="26">
+        <f>AVERAGE(E1050:E1102)</f>
+        <v>43.075471698113205</v>
+      </c>
+      <c r="F1669" s="26"/>
+      <c r="G1669" s="26">
+        <f>AVERAGE(G1050:G1102)</f>
+        <v>37.433962264150942</v>
+      </c>
+      <c r="H1669" s="26"/>
+      <c r="I1669" s="26">
+        <f>AVERAGE(I1050:I1102)</f>
+        <v>56.113207547169814</v>
       </c>
       <c r="P1669" s="2"/>
       <c r="Q1669" s="2"/>
       <c r="R1669" s="2"/>
     </row>
     <row r="1670" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1670" s="16" t="s">
-        <v>1625</v>
-      </c>
-      <c r="E1670" s="20">
-        <f>(E1657/E1605)-1</f>
-        <v>-0.14814814814814814</v>
-      </c>
-      <c r="F1670" s="20"/>
-      <c r="G1670" s="20">
-        <f>(G1657/G1605)-1</f>
-        <v>-0.26666666666666672</v>
-      </c>
-      <c r="H1670" s="20"/>
-      <c r="I1670" s="20">
-        <f>(I1657/I1605)-1</f>
-        <v>-0.10909090909090913</v>
+      <c r="B1670" s="25" t="s">
+        <v>1619</v>
+      </c>
+      <c r="C1670" s="25"/>
+      <c r="D1670" s="25"/>
+      <c r="E1670" s="1" t="s">
+        <v>1620</v>
+      </c>
+      <c r="G1670" s="1" t="s">
+        <v>1621</v>
+      </c>
+      <c r="I1670" s="1" t="s">
+        <v>1622</v>
       </c>
       <c r="P1670" s="2"/>
       <c r="Q1670" s="2"/>
       <c r="R1670" s="2"/>
     </row>
     <row r="1671" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1671" s="16" t="s">
-        <v>1626</v>
-      </c>
-      <c r="E1671" s="17">
-        <f>(E1657/F1657)-1</f>
-        <v>-0.14814814814814814</v>
-      </c>
-      <c r="G1671" s="17">
-        <f>(G1657/H1657)-1</f>
-        <v>-9.2783505154639179E-2</v>
-      </c>
-      <c r="I1671" s="17">
-        <f>(I1657/J1657)-1</f>
-        <v>2.6178010471204161E-2</v>
-      </c>
+      <c r="B1671" s="1"/>
+      <c r="C1671" s="1"/>
+      <c r="D1671" s="1"/>
       <c r="P1671" s="2"/>
       <c r="Q1671" s="2"/>
       <c r="R1671" s="2"/>
     </row>
     <row r="1672" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1672" s="14"/>
+      <c r="B1672" s="1"/>
       <c r="C1672" s="1"/>
       <c r="D1672" s="1"/>
+      <c r="E1672" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1672" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1672" s="3" t="s">
+        <v>3</v>
+      </c>
       <c r="P1672" s="2"/>
       <c r="Q1672" s="2"/>
       <c r="R1672" s="2"/>
     </row>
     <row r="1673" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1673" s="14"/>
-      <c r="C1673" s="1"/>
-      <c r="D1673" s="1"/>
+      <c r="E1673" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1673" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1673" s="39" t="s">
+        <v>1623</v>
+      </c>
+      <c r="L1673" s="1" t="s">
+        <v>1624</v>
+      </c>
       <c r="P1673" s="2"/>
       <c r="Q1673" s="2"/>
       <c r="R1673" s="2"/>
     </row>
     <row r="1674" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1674" s="14"/>
-      <c r="C1674" s="1"/>
-      <c r="D1674" s="1"/>
+      <c r="A1674" s="16" t="s">
+        <v>1625</v>
+      </c>
+      <c r="E1674" s="20">
+        <f>(E1661/E1609)-1</f>
+        <v>-6.8965517241379337E-2</v>
+      </c>
+      <c r="F1674" s="20"/>
+      <c r="G1674" s="20">
+        <f>(G1661/G1609)-1</f>
+        <v>-6.6666666666666652E-2</v>
+      </c>
+      <c r="H1674" s="20"/>
+      <c r="I1674" s="20">
+        <f>(I1661/I1609)-1</f>
+        <v>0.12195121951219523</v>
+      </c>
       <c r="P1674" s="2"/>
       <c r="Q1674" s="2"/>
       <c r="R1674" s="2"/>
     </row>
     <row r="1675" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B1675" s="14"/>
-      <c r="C1675" s="1"/>
-      <c r="D1675" s="1"/>
+      <c r="A1675" s="16" t="s">
+        <v>1626</v>
+      </c>
+      <c r="E1675" s="17">
+        <f>(E1661/F1661)-1</f>
+        <v>-0.16923076923076918</v>
+      </c>
+      <c r="G1675" s="17">
+        <f>(G1661/H1661)-1</f>
+        <v>2.7522935779816571E-2</v>
+      </c>
+      <c r="I1675" s="17">
+        <f>(I1661/J1661)-1</f>
+        <v>-7.5376884422110546E-2</v>
+      </c>
       <c r="P1675" s="2"/>
       <c r="Q1675" s="2"/>
       <c r="R1675" s="2"/>
@@ -83917,7 +84121,7 @@
       <c r="Q1744" s="2"/>
       <c r="R1744" s="2"/>
     </row>
-    <row r="1745" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1745" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1745" s="14"/>
       <c r="C1745" s="1"/>
       <c r="D1745" s="1"/>
@@ -83925,7 +84129,7 @@
       <c r="Q1745" s="2"/>
       <c r="R1745" s="2"/>
     </row>
-    <row r="1746" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1746" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1746" s="14"/>
       <c r="C1746" s="1"/>
       <c r="D1746" s="1"/>
@@ -83933,7 +84137,7 @@
       <c r="Q1746" s="2"/>
       <c r="R1746" s="2"/>
     </row>
-    <row r="1747" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1747" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1747" s="14"/>
       <c r="C1747" s="1"/>
       <c r="D1747" s="1"/>
@@ -83941,181 +84145,213 @@
       <c r="Q1747" s="2"/>
       <c r="R1747" s="2"/>
     </row>
-    <row r="1748" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1748" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B1748" s="14"/>
-      <c r="C1748" s="14"/>
-      <c r="D1748" s="14"/>
+      <c r="C1748" s="1"/>
+      <c r="D1748" s="1"/>
       <c r="P1748" s="2"/>
       <c r="Q1748" s="2"/>
       <c r="R1748" s="2"/>
     </row>
-    <row r="1749" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1749" s="14" t="s">
-        <v>1618</v>
-      </c>
-      <c r="C1749" s="14"/>
-      <c r="D1749" s="14"/>
-      <c r="E1749" s="26">
-        <f>AVERAGE(E1047:E1099)</f>
-        <v>42.490566037735846</v>
-      </c>
-      <c r="F1749" s="26"/>
-      <c r="G1749" s="26">
-        <f>AVERAGE(G1047:G1099)</f>
-        <v>37.641509433962263</v>
-      </c>
-      <c r="H1749" s="26"/>
-      <c r="I1749" s="26">
-        <f>AVERAGE(I1047:I1099)</f>
-        <v>56.320754716981135</v>
-      </c>
-      <c r="M1749" s="26"/>
+    <row r="1749" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1749" s="14"/>
+      <c r="C1749" s="1"/>
+      <c r="D1749" s="1"/>
       <c r="P1749" s="2"/>
       <c r="Q1749" s="2"/>
       <c r="R1749" s="2"/>
     </row>
-    <row r="1750" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1750" s="25" t="s">
-        <v>1619</v>
-      </c>
-      <c r="C1750" s="25"/>
-      <c r="D1750" s="25"/>
-      <c r="E1750" s="1" t="s">
-        <v>1620</v>
-      </c>
-      <c r="G1750" s="1" t="s">
-        <v>1621</v>
-      </c>
-      <c r="I1750" s="1" t="s">
-        <v>1622</v>
-      </c>
+    <row r="1750" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1750" s="14"/>
+      <c r="C1750" s="1"/>
+      <c r="D1750" s="1"/>
       <c r="P1750" s="2"/>
       <c r="Q1750" s="2"/>
       <c r="R1750" s="2"/>
     </row>
-    <row r="1751" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1751" s="1"/>
+    <row r="1751" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1751" s="14"/>
       <c r="C1751" s="1"/>
       <c r="D1751" s="1"/>
       <c r="P1751" s="2"/>
       <c r="Q1751" s="2"/>
       <c r="R1751" s="2"/>
     </row>
-    <row r="1752" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="B1752" s="1"/>
-      <c r="C1752" s="1"/>
-      <c r="D1752" s="1"/>
-      <c r="E1752" s="3" t="s">
+    <row r="1752" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1752" s="14"/>
+      <c r="C1752" s="14"/>
+      <c r="D1752" s="14"/>
+      <c r="P1752" s="2"/>
+      <c r="Q1752" s="2"/>
+      <c r="R1752" s="2"/>
+    </row>
+    <row r="1753" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1753" s="14" t="s">
+        <v>1618</v>
+      </c>
+      <c r="C1753" s="14"/>
+      <c r="D1753" s="14"/>
+      <c r="E1753" s="26">
+        <f>AVERAGE(E1047:E1099)</f>
+        <v>42.490566037735846</v>
+      </c>
+      <c r="F1753" s="26"/>
+      <c r="G1753" s="26">
+        <f>AVERAGE(G1047:G1099)</f>
+        <v>37.641509433962263</v>
+      </c>
+      <c r="H1753" s="26"/>
+      <c r="I1753" s="26">
+        <f>AVERAGE(I1047:I1099)</f>
+        <v>56.320754716981135</v>
+      </c>
+      <c r="M1753" s="26"/>
+      <c r="P1753" s="2"/>
+      <c r="Q1753" s="2"/>
+      <c r="R1753" s="2"/>
+    </row>
+    <row r="1754" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1754" s="25" t="s">
+        <v>1619</v>
+      </c>
+      <c r="C1754" s="25"/>
+      <c r="D1754" s="25"/>
+      <c r="E1754" s="1" t="s">
+        <v>1620</v>
+      </c>
+      <c r="G1754" s="1" t="s">
+        <v>1621</v>
+      </c>
+      <c r="I1754" s="1" t="s">
+        <v>1622</v>
+      </c>
+      <c r="P1754" s="2"/>
+      <c r="Q1754" s="2"/>
+      <c r="R1754" s="2"/>
+    </row>
+    <row r="1755" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1755" s="1"/>
+      <c r="C1755" s="1"/>
+      <c r="D1755" s="1"/>
+      <c r="P1755" s="2"/>
+      <c r="Q1755" s="2"/>
+      <c r="R1755" s="2"/>
+    </row>
+    <row r="1756" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B1756" s="1"/>
+      <c r="C1756" s="1"/>
+      <c r="D1756" s="1"/>
+      <c r="E1756" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="G1752" s="3" t="s">
+      <c r="G1756" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I1752" s="3" t="s">
+      <c r="I1756" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="Q1752" s="1" t="s">
+      <c r="Q1756" s="1" t="s">
         <v>1624</v>
       </c>
     </row>
-    <row r="1753" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="E1753" s="3" t="s">
+    <row r="1757" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E1757" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G1753" s="3" t="s">
+      <c r="G1757" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I1753" s="39" t="s">
+      <c r="I1757" s="39" t="s">
         <v>1623</v>
       </c>
     </row>
-    <row r="1754" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1754" s="16" t="s">
+    <row r="1758" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1758" s="16" t="s">
         <v>1625</v>
       </c>
-      <c r="E1754" s="20">
+      <c r="E1758" s="20">
         <f>(E1441/E1389)-1</f>
         <v>-0.51724137931034475</v>
       </c>
-      <c r="F1754" s="20"/>
-      <c r="G1754" s="20">
+      <c r="F1758" s="20"/>
+      <c r="G1758" s="20">
         <f>(G1441/G1389)-1</f>
         <v>0</v>
       </c>
-      <c r="H1754" s="20"/>
-      <c r="I1754" s="20">
+      <c r="H1758" s="20"/>
+      <c r="I1758" s="20">
         <f>(I1441/I1389)-1</f>
         <v>0.1020408163265305</v>
       </c>
-      <c r="M1754" s="4"/>
-      <c r="N1754" s="17"/>
-      <c r="O1754" s="4"/>
-    </row>
-    <row r="1755" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1755" s="16" t="s">
+      <c r="M1758" s="4"/>
+      <c r="N1758" s="17"/>
+      <c r="O1758" s="4"/>
+    </row>
+    <row r="1759" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1759" s="16" t="s">
         <v>1626</v>
       </c>
-      <c r="E1755" s="17">
+      <c r="E1759" s="17">
         <f>(E1441/F1441)-1</f>
         <v>-0.55555555555555558</v>
       </c>
-      <c r="G1755" s="17">
+      <c r="G1759" s="17">
         <f>(G1441/H1441)-1</f>
         <v>-0.1333333333333333</v>
       </c>
-      <c r="I1755" s="17">
+      <c r="I1759" s="17">
         <f>(I1441/J1441)-1</f>
         <v>0.17391304347826098</v>
       </c>
-      <c r="P1755" s="26"/>
-      <c r="Q1755" s="26"/>
-      <c r="R1755" s="26"/>
-      <c r="S1755" s="26"/>
-    </row>
-    <row r="1756" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1756" s="16"/>
-    </row>
-    <row r="1757" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1757" s="16"/>
-    </row>
-    <row r="1758" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1758" s="16"/>
-      <c r="N1758" s="17"/>
-      <c r="O1758" s="24"/>
-    </row>
-    <row r="1759" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A1759" s="16"/>
-      <c r="P1759" s="4"/>
-      <c r="Q1759" s="4"/>
-      <c r="R1759" s="4"/>
-      <c r="S1759" s="4"/>
-      <c r="V1759" s="4"/>
-      <c r="W1759" s="4"/>
-      <c r="X1759" s="4"/>
-    </row>
-    <row r="1761" spans="6:17" x14ac:dyDescent="0.25">
-      <c r="M1761" s="17"/>
-    </row>
-    <row r="1762" spans="6:17" x14ac:dyDescent="0.25">
-      <c r="M1762" s="17"/>
-    </row>
-    <row r="1767" spans="6:17" x14ac:dyDescent="0.25">
-      <c r="N1767" s="21"/>
-      <c r="O1767" s="21"/>
-      <c r="P1767" s="21"/>
-      <c r="Q1767" s="21"/>
-    </row>
-    <row r="1769" spans="6:17" x14ac:dyDescent="0.25">
-      <c r="F1769" s="2"/>
-    </row>
-    <row r="1818" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I1818" s="2"/>
-    </row>
-    <row r="1829" spans="16:19" x14ac:dyDescent="0.25">
-      <c r="P1829" s="4"/>
-      <c r="Q1829" s="4"/>
-      <c r="R1829" s="4"/>
-      <c r="S1829" s="4"/>
+      <c r="P1759" s="26"/>
+      <c r="Q1759" s="26"/>
+      <c r="R1759" s="26"/>
+      <c r="S1759" s="26"/>
+    </row>
+    <row r="1760" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1760" s="16"/>
+    </row>
+    <row r="1761" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1761" s="16"/>
+    </row>
+    <row r="1762" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1762" s="16"/>
+      <c r="N1762" s="17"/>
+      <c r="O1762" s="24"/>
+    </row>
+    <row r="1763" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A1763" s="16"/>
+      <c r="P1763" s="4"/>
+      <c r="Q1763" s="4"/>
+      <c r="R1763" s="4"/>
+      <c r="S1763" s="4"/>
+      <c r="V1763" s="4"/>
+      <c r="W1763" s="4"/>
+      <c r="X1763" s="4"/>
+    </row>
+    <row r="1765" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M1765" s="17"/>
+    </row>
+    <row r="1766" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="M1766" s="17"/>
+    </row>
+    <row r="1771" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="N1771" s="21"/>
+      <c r="O1771" s="21"/>
+      <c r="P1771" s="21"/>
+      <c r="Q1771" s="21"/>
+    </row>
+    <row r="1773" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="F1773" s="2"/>
+    </row>
+    <row r="1822" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I1822" s="2"/>
+    </row>
+    <row r="1833" spans="16:19" x14ac:dyDescent="0.25">
+      <c r="P1833" s="4"/>
+      <c r="Q1833" s="4"/>
+      <c r="R1833" s="4"/>
+      <c r="S1833" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A927:A932" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -84130,7 +84366,7 @@
   <pageSetup orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <ignoredErrors>
-    <ignoredError sqref="E1749:I1749 E1665:I1665" formulaRange="1"/>
+    <ignoredError sqref="E1753:I1753 E1669:I1669" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -84219,48 +84455,48 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="30">
-        <f>Data!A1657</f>
-        <v>46275</v>
+        <f>Data!A1661</f>
+        <v>46303</v>
       </c>
       <c r="B7" s="27">
-        <f>Data!E1657</f>
-        <v>23</v>
+        <f>Data!E1661</f>
+        <v>27</v>
       </c>
       <c r="C7" s="27">
-        <f>Data!G1657</f>
-        <v>22</v>
+        <f>Data!G1661</f>
+        <v>28</v>
       </c>
       <c r="D7" s="27">
-        <f>Data!I1657</f>
-        <v>49</v>
+        <f>Data!I1661</f>
+        <v>46</v>
       </c>
       <c r="E7" s="54">
-        <f>Data!M1657</f>
-        <v>11</v>
+        <f>Data!M1661</f>
+        <v>17</v>
       </c>
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="30">
-        <f>Data!A1656</f>
-        <v>46268</v>
+        <f>Data!A1660</f>
+        <v>46296</v>
       </c>
       <c r="B8" s="27">
-        <f>Data!E1656</f>
-        <v>22</v>
+        <f>Data!E1660</f>
+        <v>23</v>
       </c>
       <c r="C8" s="27">
-        <f>Data!G1656</f>
-        <v>20</v>
+        <f>Data!G1660</f>
+        <v>39</v>
       </c>
       <c r="D8" s="27">
-        <f>Data!I1656</f>
-        <v>32</v>
+        <f>Data!I1660</f>
+        <v>44</v>
       </c>
       <c r="E8" s="54">
-        <f>Data!M1656</f>
-        <v>12</v>
+        <f>Data!M1660</f>
+        <v>16</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
@@ -85125,7 +85361,7 @@
   <sheetData>
     <row r="5" spans="4:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D5" s="43" t="s">
-        <v>1693</v>
+        <v>1697</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>2</v>
@@ -85139,10 +85375,10 @@
         <v>1635</v>
       </c>
       <c r="E6" s="50">
-        <v>-0.26700000000000002</v>
+        <v>-6.7000000000000004E-2</v>
       </c>
       <c r="F6" s="51">
-        <v>-0.109</v>
+        <v>0.122</v>
       </c>
     </row>
     <row r="7" spans="4:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -85150,10 +85386,10 @@
         <v>1636</v>
       </c>
       <c r="E7" s="57">
-        <v>-9.2999999999999999E-2</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="F7" s="52">
-        <v>2.5999999999999999E-2</v>
+        <v>-7.4999999999999997E-2</v>
       </c>
     </row>
   </sheetData>
@@ -85163,6 +85399,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A79C55AAF501CD48B02588050A46B66A" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cfbbb72a77ddc149ae5429f8aad3bc86">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="e5e636eb-adfb-4590-8a37-683d3312c821" xmlns:ns3="8f98163f-4713-4d38-9764-55bef18e0fec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8aeff91eee669ee1a07d9e9975fcff3e" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -85396,7 +85641,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -85411,16 +85656,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EBCAC0B-2B80-451C-BD84-7EB5955C62C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB4B7DC8-DDD3-4AA6-9799-A9D62D6C970F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -85440,7 +85684,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B7BED19-AFAA-4C03-A209-8A99D3535EE8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -85452,14 +85696,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EBCAC0B-2B80-451C-BD84-7EB5955C62C8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{ed5b36e7-01ee-4ebc-867e-e03cfa0d4697}" enabled="0" method="" siteId="{ed5b36e7-01ee-4ebc-867e-e03cfa0d4697}" removed="1"/>

</xml_diff>